<commit_message>
Update spec check with Rongchang written confirmation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RV8phZgs8UNN3S8zYwTPRj
</commit_message>
<xml_diff>
--- a/analysis/Spec_check_offered_positions.xlsx
+++ b/analysis/Spec_check_offered_positions.xlsx
@@ -911,12 +911,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>CuSn12 centrifugal, 40 days</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Confirmed 23.10 in writing: machining per drawing; CuSn12 Sn 11–13% (not ZCuSn10Pb1/P1); same-heat test bar chemistry+spectrum. Open: mech. properties + heat No. on 3.1 cert → put in contract</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1031,12 +1031,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Unit 100, 40 days</t>
+          <t>Confirmed 23.10: CuZn35Al1 (≈ZCuZn35Al2Mn2Fe1, not H62); blank 5.5 mm; laser marking OK. Open: stand/shaft numbers from customer BEFORE order</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1071,12 +1071,12 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Unit 160</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Confirmed 23.10: CuZn35Al1; blank 5.5 mm; machining per drawing</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1231,12 +1231,12 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Unit 450</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Confirmed 23.10: CuZn35Al1; blank 8 mm; machining per drawing</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Unit 120</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Confirmed 23.10: CuZn35Al1; blank 5 mm; machining per drawing (grinding incl.)</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1311,12 +1311,12 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Unit 200</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Confirmed 23.10: CuZn35Al1; blank 6 mm; machining per drawing (grinding incl.)</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update spec check with Jiangxu confirmation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RV8phZgs8UNN3S8zYwTPRj
</commit_message>
<xml_diff>
--- a/analysis/Spec_check_offered_positions.xlsx
+++ b/analysis/Spec_check_offered_positions.xlsx
@@ -951,12 +951,12 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Price 5,000 for 33+34 incl. VAT</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>Confirmed 23.10: material per drawing (1050A), material cert, tolerances per drawing; marking OK. Asks for 3D models</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -991,12 +991,12 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>same</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+          <t>same as 33</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1111,17 +1111,17 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Snap ring included; ~30 days</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>Confirmed 23.10: 45# steel instead of St50K, snap ring included; marking OK</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Ask material: if 45# used instead of St50K, get customer OK</t>
+          <t>Get customer approval for 45# (C45) instead of St50K (E295)</t>
         </is>
       </c>
     </row>
@@ -1151,17 +1151,17 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Snap ring included</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>same as 38</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>same</t>
+          <t>Get customer approval for 45# (C45) instead of St50K (E295)</t>
         </is>
       </c>
     </row>
@@ -1191,17 +1191,17 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Snap ring included</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>same as 38</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>same</t>
+          <t>Get customer approval for 45# (C45) instead of St50K (E295)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update spec check with Kaienbo confirmation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RV8phZgs8UNN3S8zYwTPRj
</commit_message>
<xml_diff>
--- a/analysis/Spec_check_offered_positions.xlsx
+++ b/analysis/Spec_check_offered_positions.xlsx
@@ -751,7 +751,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>KMT20 in stock</t>
+          <t>Confirmed 23.10: dimensions per SKF; 45# steel with material cert; incl. 13% VAT. Open: locking pins (KMT type) not explicitly confirmed; stock/lead time due 24.10</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Confirm KMT type (locking pins), not KM + washer</t>
+          <t>Confirm KMT type with locking pins + stock</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>KMT24 in stock</t>
+          <t>Confirmed 23.10: dimensions per SKF; 45# steel with material cert; incl. 13% VAT. Open: locking pins (KMT type) not explicitly confirmed; stock/lead time due 24.10</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>same</t>
+          <t>Confirm KMT type with locking pins + stock</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>KMT28 in stock</t>
+          <t>Confirmed 23.10: dimensions per SKF; 45# steel with material cert; incl. 13% VAT. Open: locking pins (KMT type) not explicitly confirmed; stock/lead time due 24.10</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>same</t>
+          <t>Confirm KMT type with locking pins + stock</t>
         </is>
       </c>
     </row>
@@ -871,17 +871,17 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>KMT32 in stock</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>FIX</t>
+          <t>Confirmed 23.10: dimensions per SKF; 45# steel with material cert; incl. 13% VAT; KMT32 = M160×3 (standard). Open: locking pins (KMT type) not explicitly confirmed; stock/lead time due 24.10</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Confirm their KMT32 is M160×3 (standard); correct our RFQ/tracker</t>
+          <t>Confirm KMT type with locking pins + stock</t>
         </is>
       </c>
     </row>

</xml_diff>